<commit_message>
Bake latest Wave Tracker V2 data into the tool as built-in snapshot
Verified the existing parser reads the four updated workbooks correctly (sheet
names PP-01.., Management Tracker; cell layout B4/B5 + log rows 13-72 + ISSUES
unchanged). Replaced the bundled xlsx in assets/ with the latest files and
regenerated the WAVES_DATA snapshot (lib-3.js) from them, so the dashboard shows
current numbers immediately on open without any upload.

Rebuilt manifest/bundle/standalone/preview from the updated assets. Verified the
embedded snapshot, embedded xlsx, and detectRole-enabled parser all match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F4ez9fqQhzAbjYKLodyiqU
</commit_message>
<xml_diff>
--- a/waves/assets/ppFile.xlsx
+++ b/waves/assets/ppFile.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a.aalamri\Desktop\Waves Tracker\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E657806-9068-4080-A320-6B6255557EFC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBADDD11-6ED0-4E17-BD95-5040A33799A2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19160" windowHeight="7410" tabRatio="768" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="19160" windowHeight="7410" tabRatio="768" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="460" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="464" uniqueCount="127">
   <si>
     <t>رقم المشروع</t>
   </si>
@@ -427,6 +427,12 @@
   </si>
   <si>
     <t>اتم استلام متطلبات ال tco من مدير المشروع</t>
+  </si>
+  <si>
+    <t>تم الرفع</t>
+  </si>
+  <si>
+    <t>لا يوجد شيئ</t>
   </si>
 </sst>
 </file>
@@ -1871,7 +1877,7 @@
       </c>
       <c r="E5" s="5" t="str">
         <f>IFERROR(LOOKUP(2,1/('PP-01'!C13:C72&lt;&gt;""),'PP-01'!C13:C72),"—")</f>
-        <v>3 - Affordability Estimate</v>
+        <v>4 - Tender Pack Development</v>
       </c>
       <c r="F5" s="5" t="str">
         <f>IFERROR(LOOKUP(2,1/('PP-01'!D13:D72&lt;&gt;""),'PP-01'!D13:D72),"—")</f>
@@ -1879,15 +1885,15 @@
       </c>
       <c r="G5" s="6" t="str">
         <f>IFERROR(LOOKUP(2,1/('PP-01'!E13:E72&lt;&gt;""),'PP-01'!E13:E72),"—")</f>
-        <v>بانتظار ردود الشركات على طلبات الحصول على المعلومات (RFI) المرسل من قبل مدير المشروع</v>
+        <v>تم الرفع</v>
       </c>
       <c r="H5" s="4" t="str">
         <f>IFERROR(LOOKUP(2,1/('PP-01'!F13:F72&lt;&gt;""),'PP-01'!F13:F72),"—")</f>
-        <v>لا يوجد اجتماع check-out</v>
+        <v>لا يوجد شيئ</v>
       </c>
       <c r="I5" s="58" t="str">
         <f>IFERROR(LOOKUP(2,1/('PP-01'!G13:G72&lt;&gt;""),'PP-01'!G13:G72),"—")</f>
-        <v>على المسار</v>
+        <v xml:space="preserve">متأخر </v>
       </c>
     </row>
     <row r="6" spans="1:9" ht="101.5" x14ac:dyDescent="0.35">
@@ -6475,7 +6481,7 @@
       </c>
       <c r="B8" s="94" t="str">
         <f>IFERROR(LOOKUP(2,1/(C13:C72&lt;&gt;""),C13:C72),"—")</f>
-        <v>3 - Affordability Estimate</v>
+        <v>4 - Tender Pack Development</v>
       </c>
       <c r="C8" s="92"/>
       <c r="D8" s="92"/>
@@ -6493,7 +6499,7 @@
       </c>
       <c r="B9" s="97">
         <f>IFERROR(LOOKUP(2,1/(B13:B72&lt;&gt;""),B13:B72),"—")</f>
-        <v>46187</v>
+        <v>46195</v>
       </c>
       <c r="C9" s="98"/>
       <c r="D9" s="98"/>
@@ -6511,7 +6517,7 @@
       </c>
       <c r="B10" s="89" t="str">
         <f>IFERROR(INDEX(E13:E72,MATCH(MAX(B13:B72),B13:B72,0)),"—")</f>
-        <v>بانتظار ردود الشركات على طلبات الحصول على المعلومات (RFI) المرسل من قبل مدير المشروع</v>
+        <v>تم الرفع</v>
       </c>
       <c r="C10" s="90"/>
       <c r="D10" s="90"/>
@@ -6716,12 +6722,22 @@
       <c r="A20" s="16">
         <v>8</v>
       </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="18"/>
+      <c r="B20" s="62">
+        <v>46195</v>
+      </c>
+      <c r="C20" s="18" t="s">
+        <v>102</v>
+      </c>
       <c r="D20" s="18"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="14"/>
+      <c r="E20" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="F20" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="G20" s="14" t="s">
+        <v>56</v>
+      </c>
     </row>
     <row r="21" spans="1:7" ht="36" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="16">

</xml_diff>